<commit_message>
Daily slate 2026-07-06 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-29.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-29.xlsx
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>13</v>
+        <v>56</v>
       </c>
       <c r="E3" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="F3" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="G3" t="n">
-        <v>69.2</v>
+        <v>57.1</v>
       </c>
     </row>
     <row r="4">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>303</v>
+        <v>325</v>
       </c>
       <c r="E4" t="n">
-        <v>153</v>
+        <v>166</v>
       </c>
       <c r="F4" t="n">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="G4" t="n">
-        <v>50.5</v>
+        <v>51.1</v>
       </c>
     </row>
     <row r="5">
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G5" t="n">
-        <v>100</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="6">
@@ -613,16 +613,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>243</v>
+        <v>265</v>
       </c>
       <c r="E7" t="n">
-        <v>132</v>
+        <v>147</v>
       </c>
       <c r="F7" t="n">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="G7" t="n">
-        <v>54.3</v>
+        <v>55.5</v>
       </c>
     </row>
     <row r="8">
@@ -642,16 +642,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="E8" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F8" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G8" t="n">
-        <v>54.5</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="9">
@@ -671,16 +671,16 @@
         </is>
       </c>
       <c r="D9" t="n">
+        <v>32</v>
+      </c>
+      <c r="E9" t="n">
         <v>19</v>
       </c>
-      <c r="E9" t="n">
-        <v>12</v>
-      </c>
       <c r="F9" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="G9" t="n">
-        <v>63.2</v>
+        <v>59.4</v>
       </c>
     </row>
     <row r="10">
@@ -700,16 +700,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>94</v>
+        <v>171</v>
       </c>
       <c r="E10" t="n">
-        <v>70</v>
+        <v>129</v>
       </c>
       <c r="F10" t="n">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="G10" t="n">
-        <v>74.5</v>
+        <v>75.40000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -729,16 +729,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1192</v>
+        <v>1404</v>
       </c>
       <c r="E11" t="n">
-        <v>765</v>
+        <v>858</v>
       </c>
       <c r="F11" t="n">
-        <v>427</v>
+        <v>546</v>
       </c>
       <c r="G11" t="n">
-        <v>64.2</v>
+        <v>61.1</v>
       </c>
     </row>
     <row r="12">
@@ -758,16 +758,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>533</v>
+        <v>687</v>
       </c>
       <c r="E12" t="n">
-        <v>230</v>
+        <v>261</v>
       </c>
       <c r="F12" t="n">
-        <v>303</v>
+        <v>426</v>
       </c>
       <c r="G12" t="n">
-        <v>43.2</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13">
@@ -787,16 +787,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E13" t="n">
         <v>42</v>
       </c>
       <c r="F13" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G13" t="n">
-        <v>50</v>
+        <v>48.8</v>
       </c>
     </row>
     <row r="14">
@@ -816,16 +816,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>473</v>
+        <v>500</v>
       </c>
       <c r="E14" t="n">
-        <v>129</v>
+        <v>142</v>
       </c>
       <c r="F14" t="n">
-        <v>344</v>
+        <v>358</v>
       </c>
       <c r="G14" t="n">
-        <v>27.3</v>
+        <v>28.4</v>
       </c>
     </row>
     <row r="15">
@@ -845,16 +845,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>619</v>
+        <v>725</v>
       </c>
       <c r="E15" t="n">
-        <v>96</v>
+        <v>128</v>
       </c>
       <c r="F15" t="n">
-        <v>523</v>
+        <v>597</v>
       </c>
       <c r="G15" t="n">
-        <v>15.5</v>
+        <v>17.7</v>
       </c>
     </row>
     <row r="16">
@@ -874,16 +874,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>803</v>
+        <v>908</v>
       </c>
       <c r="E16" t="n">
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="F16" t="n">
-        <v>703</v>
+        <v>783</v>
       </c>
       <c r="G16" t="n">
-        <v>12.5</v>
+        <v>13.8</v>
       </c>
     </row>
     <row r="17">
@@ -903,16 +903,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4602</v>
+        <v>5188</v>
       </c>
       <c r="E17" t="n">
-        <v>862</v>
+        <v>921</v>
       </c>
       <c r="F17" t="n">
-        <v>3740</v>
+        <v>4267</v>
       </c>
       <c r="G17" t="n">
-        <v>18.7</v>
+        <v>17.8</v>
       </c>
     </row>
   </sheetData>
@@ -1450,52 +1450,52 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>74.5</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="C7" t="n">
-        <v>94</v>
+        <v>171</v>
       </c>
       <c r="D7" t="n">
-        <v>64.2</v>
+        <v>61.1</v>
       </c>
       <c r="E7" t="n">
-        <v>1192</v>
+        <v>1404</v>
       </c>
       <c r="F7" t="n">
-        <v>43.2</v>
+        <v>38</v>
       </c>
       <c r="G7" t="n">
-        <v>533</v>
+        <v>687</v>
       </c>
       <c r="H7" t="n">
-        <v>50</v>
+        <v>48.8</v>
       </c>
       <c r="I7" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="J7" t="n">
-        <v>27.3</v>
+        <v>28.4</v>
       </c>
       <c r="K7" t="n">
-        <v>473</v>
+        <v>500</v>
       </c>
       <c r="L7" t="n">
-        <v>15.5</v>
+        <v>17.7</v>
       </c>
       <c r="M7" t="n">
-        <v>619</v>
+        <v>725</v>
       </c>
       <c r="N7" t="n">
-        <v>12.5</v>
+        <v>13.8</v>
       </c>
       <c r="O7" t="n">
-        <v>803</v>
+        <v>908</v>
       </c>
       <c r="P7" t="n">
-        <v>18.7</v>
+        <v>17.8</v>
       </c>
       <c r="Q7" t="n">
-        <v>4602</v>
+        <v>5188</v>
       </c>
       <c r="R7" t="n">
         <v>65.8</v>
@@ -1504,43 +1504,43 @@
         <v>38</v>
       </c>
       <c r="T7" t="n">
-        <v>50.5</v>
+        <v>51.1</v>
       </c>
       <c r="U7" t="n">
-        <v>303</v>
+        <v>325</v>
       </c>
       <c r="W7" t="n">
         <v>0</v>
       </c>
       <c r="X7" t="n">
-        <v>54.5</v>
+        <v>45.9</v>
       </c>
       <c r="Y7" t="n">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="Z7" t="n">
-        <v>69.2</v>
+        <v>57.1</v>
       </c>
       <c r="AA7" t="n">
-        <v>13</v>
+        <v>56</v>
       </c>
       <c r="AB7" t="n">
-        <v>100</v>
+        <v>37.5</v>
       </c>
       <c r="AC7" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="AD7" t="n">
-        <v>54.3</v>
+        <v>55.5</v>
       </c>
       <c r="AE7" t="n">
-        <v>243</v>
+        <v>265</v>
       </c>
       <c r="AF7" t="n">
-        <v>63.2</v>
+        <v>59.4</v>
       </c>
       <c r="AG7" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>